<commit_message>
RESHIPPED (task236): rubric, the asks' filed-rule devices (the preliminary reports, the 28 June boundary review, the cut-off, blank and 0000 addresses, residents of other states) replaced by the gateway's person matching (a specimen's preliminary and final under two keys, an infant under its mother's key, a birthday's one-year rise) and a week 36 preliminary sent without the address from a requesting service next door; the call's rows and every other file byte-identical to the shipped pack
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/task236/golden/influenza_testing_break_flags_week36_2027.xlsx
+++ b/task236/golden/influenza_testing_break_flags_week36_2027.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="53">
   <si>
     <t>Week 36 of 2027 (6 to 12 September): testing-change break flags on four notified series, Far North, Metropolitan South, Metropolitan West, South Coast</t>
   </si>
@@ -163,7 +163,10 @@
     <t>Cases: CDB-FLU-03 section 2, built from the gateway's results. A person's positive results collected within 14 days of the first positive specimen are one case, counted in the report week of that specimen and notified when the first result reporting influenza reached the gateway, preliminary or final.</t>
   </si>
   <si>
-    <t>Regions: residential postcode under the concordance in force at the report (the postcodes moved on 28 June 2027 counted in their new regions for the whole season); cases with no residential postcode (blank, or 0000 at Northgate Diagnostics and Southern Districts Pathology) in the region of the requesting service's postcode; residents of other states not counted.</t>
+    <t>People: a specimen's preliminary and final reports that the gateway keyed to two people are one person, with that person's later results under either key; an infant whose results came under its mother's key is its own case. An age one year higher on a later specimen is the same person after a birthday.</t>
+  </si>
+  <si>
+    <t>Regions: the residential postcode recorded on any of the case's results (a preliminary sent without the address is placed by its final report), under the concordance in force at the report (the postcodes moved on 28 June 2027 counted in their new regions for the whole season); cases with no residential postcode on any result (blank, or 0000 at Northgate Diagnostics and Southern Districts Pathology) in the region of the requesting service's postcode; residents of other states not counted.</t>
   </si>
   <si>
     <t>Cut-off: cases notified by 09:00 on Monday 13 September 2027 (23:00 UTC on Sunday 12 September). Week 36 fills in after the cut-off; later notifications are counted from the week 37 report.</t>
@@ -902,7 +905,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="125" customWidth="1" min="1" max="1"/>
@@ -943,6 +946,11 @@
         <v>51</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>